<commit_message>
Altera decisões e remove template colaboradores teste
</commit_message>
<xml_diff>
--- a/relatorio_vr_072026.xlsx
+++ b/relatorio_vr_072026.xlsx
@@ -37,7 +37,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -64,11 +64,6 @@
         <fgColor rgb="00F8C9C4"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -82,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -93,10 +88,6 @@
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -462,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -574,30 +565,30 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>003</t>
+          <t>002</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Carla Mendes</t>
+          <t>Bruno Carvalho</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>770</v>
+        <v>570</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>616</v>
+        <v>456</v>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
@@ -605,49 +596,49 @@
         </is>
       </c>
       <c r="I3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
+        <v>13.64</v>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>ALERTA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>003</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Diego Santos</t>
+          <t>Carla Mendes</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>300</v>
+        <v>770</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>60</v>
+        <v>154</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>240</v>
+        <v>616</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Experiência (50%)</t>
+          <t>Integral (100%)</t>
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>9.09</v>
+        <v>0</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -658,72 +649,72 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>005</t>
+          <t>004</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Fernanda Costa</t>
+          <t>Diego Santos</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Financeiro</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>510</v>
+        <v>300</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>102</v>
+        <v>60</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>408</v>
+        <v>240</v>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Integral (100%)</t>
+          <t>Experiência (50%)</t>
         </is>
       </c>
       <c r="I5" s="4" t="n">
-        <v>22.73</v>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>ALERTA</t>
+        <v>9.09</v>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>007</t>
+          <t>005</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Helena Nunes</t>
+          <t>Fernanda Costa</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Comercial</t>
+          <t>Financeiro</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>660</v>
+        <v>510</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>132</v>
+        <v>102</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>528</v>
+        <v>408</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -731,23 +722,23 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
+        <v>22.73</v>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>ALERTA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>008</t>
+          <t>006</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Igor Ferreira</t>
+          <t>Gabriel Rocha</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -756,16 +747,16 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>630</v>
+        <v>735</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>126</v>
+        <v>147</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>504</v>
+        <v>588</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -773,49 +764,49 @@
         </is>
       </c>
       <c r="I7" s="4" t="n">
-        <v>18.18</v>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>ALERTA</t>
+        <v>4.55</v>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>009</t>
+          <t>007</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Julia Alves</t>
+          <t>Helena Nunes</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>RH</t>
+          <t>Comercial</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>315</v>
+        <v>660</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>63</v>
+        <v>132</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>252</v>
+        <v>528</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Experiência (50%)</t>
+          <t>Integral (100%)</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>4.55</v>
+        <v>0</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -826,30 +817,30 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>010</t>
+          <t>008</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Lucas Martins</t>
+          <t>Igor Ferreira</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>660</v>
+        <v>630</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>528</v>
+        <v>504</v>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
@@ -857,49 +848,49 @@
         </is>
       </c>
       <c r="I9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
+        <v>18.18</v>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>ALERTA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>011</t>
+          <t>009</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Mariana Souza</t>
+          <t>Julia Alves</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Financeiro</t>
+          <t>RH</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>600</v>
+        <v>315</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>120</v>
+        <v>63</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>480</v>
+        <v>252</v>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Integral (100%)</t>
+          <t>Experiência (50%)</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>9.09</v>
+        <v>4.55</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -910,30 +901,30 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>012</t>
+          <t>010</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Nicolas Prado</t>
+          <t>Lucas Martins</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>TI</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>560</v>
+        <v>660</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>448</v>
+        <v>528</v>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
@@ -941,49 +932,49 @@
         </is>
       </c>
       <c r="I11" s="4" t="n">
-        <v>27.27</v>
-      </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>ALERTA</t>
+        <v>0</v>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>013</t>
+          <t>011</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Olivia Teixeira</t>
+          <t>Mariana Souza</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Comercial</t>
+          <t>Financeiro</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>315</v>
+        <v>600</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>252</v>
+        <v>480</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Experiência (50%)</t>
+          <t>Integral (100%)</t>
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>4.55</v>
+        <v>9.09</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -994,40 +985,166 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Nicolas Prado</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Logística</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>560</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>112</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>448</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Integral (100%)</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>27.27</v>
+      </c>
+      <c r="J13" s="6" t="inlineStr">
+        <is>
+          <t>ALERTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Olivia Teixeira</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Comercial</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>315</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>252</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Experiência (50%)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>014</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Paulo Rezende</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>RH</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D15" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E15" s="5" t="n">
         <v>660</v>
       </c>
-      <c r="F13" s="5" t="n">
+      <c r="F15" s="5" t="n">
         <v>132</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G15" s="5" t="n">
         <v>528</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Integral (100%)</t>
         </is>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="I15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Renata Gomes</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>600</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>120</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>480</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Integral (100%)</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>9.09</v>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1070,7 +1187,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -1080,7 +1197,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>5372</v>
+        <v>6896</v>
       </c>
     </row>
     <row r="4">
@@ -1090,7 +1207,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -1110,7 +1227,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1121,7 +1238,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>08/07/2026 16:15:15</t>
+          <t>08/07/2026 17:06:29</t>
         </is>
       </c>
     </row>
@@ -1136,14 +1253,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1174,77 +1291,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>001</t>
-        </is>
-      </c>
-      <c r="C2" s="8" t="inlineStr">
-        <is>
-          <t>Bruno Carvalho</t>
-        </is>
-      </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>matricula</t>
-        </is>
-      </c>
-      <c r="E2" s="9" t="inlineStr">
-        <is>
-          <t>matrícula duplicada; já encontrada na linha 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>006</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Gabriel Rocha</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>dias_trabalhados</t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>dias_trabalhados (23) não pode ser maior que dias_uteis_mes (22).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="n">
-        <v>16</v>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>015</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>nome</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>nome é obrigatório e não pode estar vazio.</t>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Nenhum erro de validação encontrado.</t>
         </is>
       </c>
     </row>

</xml_diff>